<commit_message>
Verifica settimanale: 16 duplicati marcati, 26 upgrade doppio controllo
Completata la verifica di qualita sui file .xlsx in /output (3 file, 48
righe esaminate in deduplica globale). 26 record con doppio controllo
WebSearch indipendente positivo passano a 'VERIFICATA AI - doppio
controllo (31/08/2026)'; 6 record con esito ambiguo/non confermato
restano 'DA VERIFICARE UMANAMENTE' senza modifiche. Nessun record e'
mai trattato come dato definitivo senza controllo umano finale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158TzxJdksXSnffhmC7YjQN
</commit_message>
<xml_diff>
--- a/output/2026-08-31_08_Italia_Toscana_Cleaning.xlsx
+++ b/output/2026-08-31_08_Italia_Toscana_Cleaning.xlsx
@@ -487,7 +487,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Oltre 30 anni di attività, progettazione/installazione impianti di aspirazione industriale, depolverizzazione, filtri a maniche/cartucce/carboni attivi.</t>
@@ -495,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -532,7 +531,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -569,7 +568,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -606,7 +605,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -631,7 +630,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Rivenditore/distributore esclusivo Rotowash per FI/PO/PT/SI/AR/GR/PI/LI; tratta anche Karcher, Nilfisk, Eureka, Annovi Reverberi, Biemmedue, IPC, ITM, OMM, Wirbel.</t>
@@ -639,7 +637,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -664,7 +662,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Gruppo attivo da oltre 40 anni nella pulizia industriale/professionale; sede locale Firenze con vendita macchine e ingrosso prodotti.</t>
@@ -697,7 +694,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Noleggio, assistenza e vendita macchine pulizia civile/industriale (lavasciuga, spazzatrici, aspiratori); sede a Calenzano.</t>
@@ -705,7 +701,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -742,7 +738,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -767,7 +763,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>Oltre 30 anni di attività; noleggio/vendita macchine pulizia industriale multi-brand (Comac, CFM, Dulevo, RCM), sedi Firenze e Livorno.</t>
@@ -775,7 +770,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -837,7 +832,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>Concessionario RCM per provincie di Pistoia e Firenze; vendita/assistenza aspiratori RCM, IPC, Coynco, lavapavimenti e spazzatrici.</t>
@@ -845,7 +839,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -870,7 +864,6 @@
           <t>Cleaning</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Sede Via Zarini 136, Prato. Noleggio/vendita lavasciuga, spazzatrici, idropulitrici, lavamoquette per pulizia civile e industriale.</t>
@@ -878,7 +871,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -915,7 +908,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -952,7 +945,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -989,7 +982,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1056,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (31/08/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>